<commit_message>
Update report template Excel file to reflect recent changes
</commit_message>
<xml_diff>
--- a/report_template.xlsx
+++ b/report_template.xlsx
@@ -8,13 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sixii\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB9453C2-F8AB-4638-817C-E1BDDB159625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{319DCF6A-936E-4634-96DF-3C44F7610038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="8" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+    <externalReference r:id="rId3"/>
+    <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
+    <externalReference r:id="rId6"/>
+    <externalReference r:id="rId7"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1741,7 +1749,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.41718054551552469"/>
+          <c:y val="0.17562201957956836"/>
+          <c:w val="0.57992558722489385"/>
+          <c:h val="0.60033716141213578"/>
+        </c:manualLayout>
+      </c:layout>
       <c:doughnutChart>
         <c:varyColors val="1"/>
         <c:ser>
@@ -2133,8 +2151,8 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="3.9168637685040864E-2"/>
-          <c:y val="0.26897378961367174"/>
+          <c:x val="0.16976095114889231"/>
+          <c:y val="0.14197369573212379"/>
           <c:w val="0.66974866985455206"/>
           <c:h val="0.61293251875567556"/>
         </c:manualLayout>
@@ -6876,15 +6894,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>40822</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:rowOff>157842</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
+      <xdr:colOff>48442</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
+      <xdr:rowOff>1632</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7028,6 +7046,84 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="All_Socials"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Facebook"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Instagram"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="LinkedIn"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="TikTok"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Twitter"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -7392,67 +7488,67 @@
         <v>9</v>
       </c>
       <c r="C5" s="7" t="e">
-        <f>COUNTIF(#REF!,"positive")</f>
-        <v>#REF!</v>
+        <f>COUNTIF([1]All_Socials!D:D,"Positive")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="D5" s="8" t="e">
         <f>C5/C8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>9</v>
       </c>
       <c r="G5" s="4" t="e">
-        <f>COUNTIFS(#REF!,"positive")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([2]Facebook!D:D,"Positive")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="H5" s="9" t="e">
         <f>G5/G8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J5" s="7" t="s">
         <v>9</v>
       </c>
       <c r="K5" s="4" t="e">
-        <f>COUNTIFS(#REF!,"positive")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([3]Instagram!D:D,"Positive")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="L5" s="9" t="e">
         <f>K5/K8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="N5" s="7" t="s">
         <v>9</v>
       </c>
       <c r="O5" s="4" t="e">
-        <f>COUNTIFS(#REF!,"Positive")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([4]LinkedIn!D:D,"Positive")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="P5" s="9" t="e">
         <f>O5/O8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="R5" s="7" t="s">
         <v>9</v>
       </c>
       <c r="S5" s="4" t="e">
-        <f>COUNTIFS(#REF!,"Positive")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([5]TikTok!D:D,"Positive")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="T5" s="9" t="e">
         <f>S5/S8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="V5" s="7" t="s">
         <v>9</v>
       </c>
       <c r="W5" s="4" t="e">
-        <f>COUNTIFS(#REF!,"positive")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([6]Twitter!D:D,"Positive")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="X5" s="9" t="e">
         <f>W5/W8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="6" spans="1:24">
@@ -7460,67 +7556,67 @@
         <v>10</v>
       </c>
       <c r="C6" s="7" t="e">
-        <f>COUNTIF(#REF!,"neutral")</f>
-        <v>#REF!</v>
+        <f>COUNTIF([1]All_Socials!D:D,"Neutral")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="D6" s="8" t="e">
         <f>C6/C8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>10</v>
       </c>
       <c r="G6" s="4" t="e">
-        <f>COUNTIFS(#REF!,"neutral")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([2]Facebook!D:D,"Neutral")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="H6" s="9" t="e">
         <f>G6/G8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="4" t="e">
-        <f>COUNTIFS(#REF!,"neutral")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([3]Instagram!D:D,"Neutral")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="L6" s="9" t="e">
         <f>K6/K8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="N6" s="7" t="s">
         <v>10</v>
       </c>
       <c r="O6" s="4" t="e">
-        <f>COUNTIFS(#REF!,"Neutral")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([4]LinkedIn!D:D,"Neutral")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="P6" s="9" t="e">
         <f>O6/O8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="R6" s="7" t="s">
         <v>10</v>
       </c>
       <c r="S6" s="4" t="e">
-        <f>COUNTIFS(#REF!,"Neutral")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([5]TikTok!D:D,"Neutral")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="T6" s="9" t="e">
         <f>S6/S8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="V6" s="7" t="s">
         <v>10</v>
       </c>
       <c r="W6" s="4" t="e">
-        <f>COUNTIFS(#REF!,"Neutral")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([6]Twitter!D:D,"Neutral")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="X6" s="9" t="e">
         <f>W6/W8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="18" thickBot="1">
@@ -7528,67 +7624,67 @@
         <v>11</v>
       </c>
       <c r="C7" s="10" t="e">
-        <f>COUNTIF(#REF!,"Negative")</f>
-        <v>#REF!</v>
+        <f>COUNTIF([1]All_Socials!D:D,"Negative")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="D7" s="11" t="e">
         <f>C7/C8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>11</v>
       </c>
       <c r="G7" s="12" t="e">
-        <f>COUNTIFS(#REF!,"negative")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([2]Facebook!D:D,"Negative")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="H7" s="13" t="e">
         <f>G7/G8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>11</v>
       </c>
       <c r="K7" s="12" t="e">
-        <f>COUNTIFS(#REF!,"Negative ")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([3]Instagram!D:D,"Negative")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="L7" s="13" t="e">
         <f>K7/K8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="N7" s="10" t="s">
         <v>11</v>
       </c>
       <c r="O7" s="4" t="e">
-        <f>COUNTIFS(#REF!,"Negative")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([4]LinkedIn!D:D,"Negative")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="P7" s="13" t="e">
         <f>O7/O8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="R7" s="10" t="s">
         <v>11</v>
       </c>
       <c r="S7" s="4" t="e">
-        <f>COUNTIFS(#REF!,"Negative")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([5]TikTok!D:D,"Negative")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="T7" s="13" t="e">
         <f>S7/S8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="V7" s="10" t="s">
         <v>11</v>
       </c>
       <c r="W7" s="4" t="e">
-        <f>COUNTIFS(#REF!,"Negative")</f>
-        <v>#REF!</v>
+        <f>COUNTIFS([6]Twitter!D:D,"Negative")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="X7" s="13" t="e">
         <f>W7/W8</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="1:24">
@@ -7597,7 +7693,7 @@
       </c>
       <c r="C8" s="14" t="e">
         <f>SUM(C5:C7)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>13</v>
@@ -7607,55 +7703,55 @@
       </c>
       <c r="G8" s="16" t="e">
         <f>SUM(G5:G7)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="H8" s="17" t="e">
         <f>SUM(H5:H7)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J8" s="18" t="s">
         <v>12</v>
       </c>
       <c r="K8" s="19" t="e">
         <f>SUM(K5:K7)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="L8" s="20" t="e">
         <f>SUM(L5:L7)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="N8" s="14" t="s">
         <v>12</v>
       </c>
       <c r="O8" s="16" t="e">
         <f>SUM(O5:O7)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="P8" s="17" t="e">
         <f>SUM(P5:P7)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="R8" s="14" t="s">
         <v>12</v>
       </c>
       <c r="S8" s="16" t="e">
         <f>SUM(S5:S7)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="T8" s="17" t="e">
         <f>SUM(T5:T7)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="V8" s="14" t="s">
         <v>12</v>
       </c>
       <c r="W8" s="16" t="e">
         <f>SUM(W5:W7)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="X8" s="17" t="e">
         <f>SUM(X5:X7)</f>
-        <v>#REF!</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="24" spans="1:18">
@@ -7730,67 +7826,49 @@
       <c r="C29" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="D29" s="32">
-        <v>1</v>
-      </c>
+      <c r="D29" s="32"/>
       <c r="F29" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="G29" s="24">
-        <v>1</v>
-      </c>
+      <c r="G29" s="24"/>
     </row>
     <row r="30" spans="1:18">
       <c r="C30" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="D30" s="32">
-        <v>1</v>
-      </c>
+      <c r="D30" s="32"/>
       <c r="F30" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="G30" s="24">
-        <v>2</v>
-      </c>
+      <c r="G30" s="24"/>
     </row>
     <row r="31" spans="1:18" ht="34.5">
       <c r="C31" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="D31" s="32">
-        <v>10</v>
-      </c>
+      <c r="D31" s="32"/>
       <c r="F31" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="G31" s="24">
-        <v>1</v>
-      </c>
+      <c r="G31" s="24"/>
     </row>
     <row r="32" spans="1:18" ht="34.5">
       <c r="F32" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="G32" s="24">
-        <v>1</v>
-      </c>
+      <c r="G32" s="24"/>
     </row>
     <row r="33" spans="6:7">
       <c r="F33" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="G33" s="24">
-        <v>1</v>
-      </c>
+      <c r="G33" s="24"/>
     </row>
     <row r="34" spans="6:7">
       <c r="F34" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="G34" s="24">
-        <v>1</v>
-      </c>
+      <c r="G34" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>